<commit_message>
docs(reports): deploy unified consolidated summary reports for build 20
</commit_message>
<xml_diff>
--- a/reports/history/android/build-20/Excel/Execution_Summary.xlsx
+++ b/reports/history/android/build-20/Excel/Execution_Summary.xlsx
@@ -525,14 +525,14 @@
         <v>518</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>99.81%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>

</xml_diff>